<commit_message>
Tighten dashboard chart layout
</commit_message>
<xml_diff>
--- a/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
+++ b/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Re67917f9fd46497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R719d8549b9c14aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="R6ceea74eb7c2417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R1c0846a9ed4c4af6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -938,13 +938,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -960,7 +960,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0e016e1768e04f54"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R220d788ab4034d5e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -968,15 +968,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>58</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -990,7 +990,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdec9bab2efa64d62"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcfac576ce5274616"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1842,7 +1842,7 @@
     <x:mergeCell ref="J9:K9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0004f69ea77848c3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc236a2125b234af1"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Move chart helpers off dashboard
</commit_message>
<xml_diff>
--- a/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
+++ b/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Ra962b896b66340de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R6d93073ccec048dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Rf8dd917e1e8e43e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R3bf669a8cfab40e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -735,7 +735,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Dashboard &amp; Metrics'!$A$42:$A$54</c:f>
+              <c:f>'90-Day Ledger'!$J$2:$J$14</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -743,7 +743,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard &amp; Metrics'!$B$42:$B$54</c:f>
+              <c:f>'90-Day Ledger'!$K$2:$K$14</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -760,7 +760,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Dashboard &amp; Metrics'!$A$42:$A$54</c:f>
+              <c:f>'90-Day Ledger'!$J$2:$J$14</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -768,7 +768,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard &amp; Metrics'!$C$42:$C$54</c:f>
+              <c:f>'90-Day Ledger'!$L$2:$L$14</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -890,7 +890,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Dashboard &amp; Metrics'!$K$42:$K$45</c:f>
+              <c:f>'90-Day Ledger'!$N$2:$N$5</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -898,7 +898,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Dashboard &amp; Metrics'!$L$42:$L$45</c:f>
+              <c:f>'90-Day Ledger'!$O$2:$O$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="0"/>
@@ -944,9 +944,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -960,7 +960,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7db66a60b8ec4cea"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ef3e45adef14150"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -968,15 +968,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -990,7 +990,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4c6eb62cb1b4342"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1ee158de29374d13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1613,220 +1613,6 @@
       <x:c r="G24" s="83"/>
       <x:c r="H24" s="83"/>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="60" t="str">
-        <x:v>Week</x:v>
-      </x:c>
-      <x:c r="B41" s="60" t="str">
-        <x:v>Planned Cumulative</x:v>
-      </x:c>
-      <x:c r="C41" s="60" t="str">
-        <x:v>Actual Cumulative</x:v>
-      </x:c>
-      <x:c r="K41" s="60" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="L41" s="60" t="str">
-        <x:v>Count</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="152" t="str">
-        <x:v>Week 1</x:v>
-      </x:c>
-      <x:c r="B42" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$8)</x:f>
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C42" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$8)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K42" s="152" t="str">
-        <x:v>SUCCESS</x:v>
-      </x:c>
-      <x:c r="L42" s="153" t="n">
-        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"SUCCESS")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="152" t="str">
-        <x:v>Week 2</x:v>
-      </x:c>
-      <x:c r="B43" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$15)</x:f>
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="C43" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$15)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K43" s="152" t="str">
-        <x:v>PARTIAL SUCCESS</x:v>
-      </x:c>
-      <x:c r="L43" s="153" t="n">
-        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"PARTIAL SUCCESS")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="152" t="str">
-        <x:v>Week 3</x:v>
-      </x:c>
-      <x:c r="B44" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$22)</x:f>
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C44" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$22)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K44" s="152" t="str">
-        <x:v>FAILURE</x:v>
-      </x:c>
-      <x:c r="L44" s="153" t="n">
-        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"FAILURE")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="152" t="str">
-        <x:v>Week 4</x:v>
-      </x:c>
-      <x:c r="B45" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$29)</x:f>
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="C45" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$29)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K45" s="152" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="L45" s="153" t="n">
-        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"PENDING")</x:f>
-        <x:v>90</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="152" t="str">
-        <x:v>Week 5</x:v>
-      </x:c>
-      <x:c r="B46" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$36)</x:f>
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="C46" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$36)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="152" t="str">
-        <x:v>Week 6</x:v>
-      </x:c>
-      <x:c r="B47" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$43)</x:f>
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="C47" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$43)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="152" t="str">
-        <x:v>Week 7</x:v>
-      </x:c>
-      <x:c r="B48" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$50)</x:f>
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="C48" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$50)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="152" t="str">
-        <x:v>Week 8</x:v>
-      </x:c>
-      <x:c r="B49" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$57)</x:f>
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="C49" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$57)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="152" t="str">
-        <x:v>Week 9</x:v>
-      </x:c>
-      <x:c r="B50" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$64)</x:f>
-        <x:v>333</x:v>
-      </x:c>
-      <x:c r="C50" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$64)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="152" t="str">
-        <x:v>Week 10</x:v>
-      </x:c>
-      <x:c r="B51" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$71)</x:f>
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="C51" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$71)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="152" t="str">
-        <x:v>Week 11</x:v>
-      </x:c>
-      <x:c r="B52" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$78)</x:f>
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="C52" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$78)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="152" t="str">
-        <x:v>Week 12</x:v>
-      </x:c>
-      <x:c r="B53" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$85)</x:f>
-        <x:v>522</x:v>
-      </x:c>
-      <x:c r="C53" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$85)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="152" t="str">
-        <x:v>Week 13</x:v>
-      </x:c>
-      <x:c r="B54" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$D$2:$D$91)</x:f>
-        <x:v>583</x:v>
-      </x:c>
-      <x:c r="C54" s="153" t="n">
-        <x:f>SUM('90-Day Ledger'!$E$2:$E$91)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -1854,7 +1640,7 @@
     <x:mergeCell ref="J9:K9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc312e08f16a47d9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e8b4f01f93144d4"/>
 </x:worksheet>
 </file>
 
@@ -1897,6 +1683,21 @@
       <x:c r="H1" s="6" t="str">
         <x:v>Workout Link</x:v>
       </x:c>
+      <x:c r="J1" s="60" t="str">
+        <x:v>Week</x:v>
+      </x:c>
+      <x:c r="K1" s="60" t="str">
+        <x:v>Planned Cumulative</x:v>
+      </x:c>
+      <x:c r="L1" s="60" t="str">
+        <x:v>Actual Cumulative</x:v>
+      </x:c>
+      <x:c r="N1" s="60" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="O1" s="60" t="str">
+        <x:v>Count</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="str">
@@ -1924,6 +1725,24 @@
       <x:c r="H2" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J2" s="152" t="str">
+        <x:v>Week 1</x:v>
+      </x:c>
+      <x:c r="K2" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$8)</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L2" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="152" t="str">
+        <x:v>SUCCESS</x:v>
+      </x:c>
+      <x:c r="O2" s="153" t="n">
+        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"SUCCESS")</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="18" t="str">
@@ -1951,6 +1770,24 @@
       <x:c r="H3" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J3" s="152" t="str">
+        <x:v>Week 2</x:v>
+      </x:c>
+      <x:c r="K3" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$15)</x:f>
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="L3" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$15)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N3" s="152" t="str">
+        <x:v>PARTIAL SUCCESS</x:v>
+      </x:c>
+      <x:c r="O3" s="153" t="n">
+        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"PARTIAL SUCCESS")</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18" t="str">
@@ -1978,6 +1815,24 @@
       <x:c r="H4" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J4" s="152" t="str">
+        <x:v>Week 3</x:v>
+      </x:c>
+      <x:c r="K4" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$22)</x:f>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="L4" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$22)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="152" t="str">
+        <x:v>FAILURE</x:v>
+      </x:c>
+      <x:c r="O4" s="153" t="n">
+        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"FAILURE")</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18" t="str">
@@ -2005,6 +1860,24 @@
       <x:c r="H5" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J5" s="152" t="str">
+        <x:v>Week 4</x:v>
+      </x:c>
+      <x:c r="K5" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$29)</x:f>
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="L5" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N5" s="152" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
+      <x:c r="O5" s="153" t="n">
+        <x:f>COUNTIF('90-Day Ledger'!$G$2:$G$91,"PENDING")</x:f>
+        <x:v>90</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18" t="str">
@@ -2032,6 +1905,17 @@
       <x:c r="H6" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J6" s="152" t="str">
+        <x:v>Week 5</x:v>
+      </x:c>
+      <x:c r="K6" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$36)</x:f>
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="L6" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$36)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="18" t="str">
@@ -2059,6 +1943,17 @@
       <x:c r="H7" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J7" s="152" t="str">
+        <x:v>Week 6</x:v>
+      </x:c>
+      <x:c r="K7" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$43)</x:f>
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="L7" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$43)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="18" t="str">
@@ -2086,6 +1981,17 @@
       <x:c r="H8" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J8" s="152" t="str">
+        <x:v>Week 7</x:v>
+      </x:c>
+      <x:c r="K8" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$50)</x:f>
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="L8" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$50)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="18" t="str">
@@ -2113,6 +2019,17 @@
       <x:c r="H9" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J9" s="152" t="str">
+        <x:v>Week 8</x:v>
+      </x:c>
+      <x:c r="K9" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$57)</x:f>
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="L9" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$57)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18" t="str">
@@ -2140,6 +2057,17 @@
       <x:c r="H10" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J10" s="152" t="str">
+        <x:v>Week 9</x:v>
+      </x:c>
+      <x:c r="K10" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$64)</x:f>
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="L10" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$64)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18" t="str">
@@ -2167,6 +2095,17 @@
       <x:c r="H11" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J11" s="152" t="str">
+        <x:v>Week 10</x:v>
+      </x:c>
+      <x:c r="K11" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$71)</x:f>
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="L11" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$71)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="18" t="str">
@@ -2194,6 +2133,17 @@
       <x:c r="H12" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J12" s="152" t="str">
+        <x:v>Week 11</x:v>
+      </x:c>
+      <x:c r="K12" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$78)</x:f>
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="L12" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$78)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18" t="str">
@@ -2221,6 +2171,17 @@
       <x:c r="H13" s="17" t="str">
         <x:v>Open workout</x:v>
       </x:c>
+      <x:c r="J13" s="152" t="str">
+        <x:v>Week 12</x:v>
+      </x:c>
+      <x:c r="K13" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$85)</x:f>
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="L13" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$85)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="18" t="str">
@@ -2247,6 +2208,17 @@
       </x:c>
       <x:c r="H14" s="17" t="str">
         <x:v>Open workout</x:v>
+      </x:c>
+      <x:c r="J14" s="152" t="str">
+        <x:v>Week 13</x:v>
+      </x:c>
+      <x:c r="K14" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$D$2:$D$91)</x:f>
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="L14" s="153" t="n">
+        <x:f>SUM('90-Day Ledger'!$E$2:$E$91)</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15">

</xml_diff>

<commit_message>
Reposition charts into dashboard gap
</commit_message>
<xml_diff>
--- a/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
+++ b/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Rf8dd917e1e8e43e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R3bf669a8cfab40e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Re0e7dd7cb8d7485c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="Racf1be165a934405"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -938,15 +938,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -960,7 +960,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ef3e45adef14150"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad262c7473c04462"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -968,15 +968,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -990,7 +990,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1ee158de29374d13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd864b5ecce8e40a6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1640,7 +1640,7 @@
     <x:mergeCell ref="J9:K9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e8b4f01f93144d4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c757c6088e64682"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Point workout links to LDS site
</commit_message>
<xml_diff>
--- a/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
+++ b/outputs/missionary_ready_90_day_tracker/missionary_ready_90_day_tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="Re0e7dd7cb8d7485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="Racf1be165a934405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard &amp; Metrics" sheetId="1" r:id="R8215071251c0456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-Day Ledger" sheetId="2" r:id="R0333c0098d4047a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -960,7 +960,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad262c7473c04462"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re71ca5b36a9e4382"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -990,7 +990,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd864b5ecce8e40a6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rce07a977fc7c4a88"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1640,7 +1640,7 @@
     <x:mergeCell ref="J9:K9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c757c6088e64682"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf831e6f1190c4e79"/>
 </x:worksheet>
 </file>
 

</xml_diff>